<commit_message>
Update trip dates to start July 25th 2026
</commit_message>
<xml_diff>
--- a/spring_hike_menu_19_people.xlsx
+++ b/spring_hike_menu_19_people.xlsx
@@ -783,7 +783,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>April 4–6, 2026  ·  Fremont → Lake Del Valle  ·  26.4 mi  ·  13 Scouts · 6 Adults  |  3 Scout cans (3 people) · 1 Scout can (4 people) · 2 Adult cans (3 people)</t>
+          <t>July 25–27, 2026  ·  Fremont → Lake Del Valle  ·  26.4 mi  ·  13 Scouts · 6 Adults  |  3 Scout cans (3 people) · 1 Scout can (4 people) · 2 Adult cans (3 people)</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Sat Apr 4</t>
+          <t>Sat Jul 25</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Sun Apr 5</t>
+          <t>Sun Jul 26</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Mon Apr 6</t>
+          <t>Mon Jul 27</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
@@ -1318,7 +1318,7 @@
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Sat Apr 4 delivered</t>
+          <t>Sat Jul 25 delivered</t>
         </is>
       </c>
       <c r="B21" s="16">
@@ -1338,7 +1338,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Sun Apr 5 delivered</t>
+          <t>Sun Jul 26 delivered</t>
         </is>
       </c>
       <c r="B22" s="17">
@@ -1358,7 +1358,7 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Mon Apr 6 delivered</t>
+          <t>Mon Jul 27 delivered</t>
         </is>
       </c>
       <c r="B23" s="16">
@@ -1706,14 +1706,14 @@
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="25" t="inlineStr">
         <is>
-          <t>SAT APR 4 — BREAKFAST (Eaten at home before driving to trailhead)</t>
+          <t>SAT JUL 25 — BREAKFAST (Eaten at home before driving to trailhead)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>SAT APR 4 — SNACKS (Handed out at trailhead)</t>
+          <t>SAT JUL 25 — SNACKS (Handed out at trailhead)</t>
         </is>
       </c>
     </row>
@@ -2199,7 +2199,7 @@
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>SAT APR 4 — LUNCH (NO COOK — trail charcuterie)</t>
+          <t>SAT JUL 25 — LUNCH (NO COOK — trail charcuterie)</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2553,7 @@
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>SAT APR 4 — DINNER (hot, communal — Star's Rest)</t>
+          <t>SAT JUL 25 — DINNER (hot, communal — Star's Rest)</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>SAT APR 4 — DESSERT (Crème Brûlée)</t>
+          <t>SAT JUL 25 — DESSERT (Crème Brûlée)</t>
         </is>
       </c>
     </row>
@@ -3195,7 +3195,7 @@
     <row r="30">
       <c r="A30" s="43" t="inlineStr">
         <is>
-          <t>SAT APR 4 — DAILY TOTAL (Per Bear Can)</t>
+          <t>SAT JUL 25 — DAILY TOTAL (Per Bear Can)</t>
         </is>
       </c>
       <c r="B30" s="43" t="n"/>
@@ -3245,7 +3245,7 @@
     <row r="31">
       <c r="A31" s="47" t="inlineStr">
         <is>
-          <t>SAT APR 4 — CALORIES DELIVERED PER PERSON</t>
+          <t>SAT JUL 25 — CALORIES DELIVERED PER PERSON</t>
         </is>
       </c>
       <c r="B31" s="47" t="n"/>
@@ -3277,7 +3277,7 @@
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>SUN APR 5 — BREAKFAST (grab &amp; go — MET-Rx Big100)</t>
+          <t>SUN JUL 26 — BREAKFAST (grab &amp; go — MET-Rx Big100)</t>
         </is>
       </c>
     </row>
@@ -3565,7 +3565,7 @@
     <row r="37" ht="24" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>SUN APR 5 — SNACKS (individual — all cans)</t>
+          <t>SUN JUL 26 — SNACKS (individual — all cans)</t>
         </is>
       </c>
     </row>
@@ -3985,7 +3985,7 @@
     <row r="44" ht="24" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>SUN APR 5 — ADULT SUPPLEMENT (Adult Cans Only)</t>
+          <t>SUN JUL 26 — ADULT SUPPLEMENT (Adult Cans Only)</t>
         </is>
       </c>
     </row>
@@ -4273,7 +4273,7 @@
     <row r="49" ht="24" customHeight="1">
       <c r="A49" s="54" t="inlineStr">
         <is>
-          <t>SUN APR 5 — LUNCH (NO COOK — chicken wraps)</t>
+          <t>SUN JUL 26 — LUNCH (NO COOK — chicken wraps)</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
     <row r="57" ht="24" customHeight="1">
       <c r="A57" s="26" t="inlineStr">
         <is>
-          <t>SUN APR 5 — DINNER (hot, communal — Maggie's Half Acre)</t>
+          <t>SUN JUL 26 — DINNER (hot, communal — Maggie's Half Acre)</t>
         </is>
       </c>
     </row>
@@ -5179,7 +5179,7 @@
     <row r="64" ht="24" customHeight="1">
       <c r="A64" s="26" t="inlineStr">
         <is>
-          <t>SUN APR 5 — DESSERT (Justin's Dark Choc PB Cups)</t>
+          <t>SUN JUL 26 — DESSERT (Justin's Dark Choc PB Cups)</t>
         </is>
       </c>
     </row>
@@ -5401,7 +5401,7 @@
     <row r="68">
       <c r="A68" s="43" t="inlineStr">
         <is>
-          <t>SUN APR 5 — DAILY TOTAL (Per Bear Can)</t>
+          <t>SUN JUL 26 — DAILY TOTAL (Per Bear Can)</t>
         </is>
       </c>
       <c r="B68" s="43" t="n"/>
@@ -5451,7 +5451,7 @@
     <row r="69">
       <c r="A69" s="47" t="inlineStr">
         <is>
-          <t>SUN APR 5 — CALORIES DELIVERED PER PERSON</t>
+          <t>SUN JUL 26 — CALORIES DELIVERED PER PERSON</t>
         </is>
       </c>
       <c r="B69" s="47" t="n"/>
@@ -5483,7 +5483,7 @@
     <row r="70" ht="24" customHeight="1">
       <c r="A70" s="26" t="inlineStr">
         <is>
-          <t>MON APR 6 — BREAKFAST (grab &amp; go — ProBar Meal)</t>
+          <t>MON JUL 27 — BREAKFAST (grab &amp; go — ProBar Meal)</t>
         </is>
       </c>
     </row>
@@ -5771,7 +5771,7 @@
     <row r="75" ht="24" customHeight="1">
       <c r="A75" s="54" t="inlineStr">
         <is>
-          <t>MON APR 6 — SNACKS (hip-belt pocket)</t>
+          <t>MON JUL 27 — SNACKS (hip-belt pocket)</t>
         </is>
       </c>
     </row>
@@ -6191,7 +6191,7 @@
     <row r="82" ht="24" customHeight="1">
       <c r="A82" s="54" t="inlineStr">
         <is>
-          <t>MON APR 6 — LUNCH (NO COOK — PB wraps)</t>
+          <t>MON JUL 27 — LUNCH (NO COOK — PB wraps)</t>
         </is>
       </c>
     </row>
@@ -6479,7 +6479,7 @@
     <row r="87">
       <c r="A87" s="43" t="inlineStr">
         <is>
-          <t>MON APR 6 — DAILY TOTAL (Per Bear Can)</t>
+          <t>MON JUL 27 — DAILY TOTAL (Per Bear Can)</t>
         </is>
       </c>
       <c r="B87" s="43" t="n"/>
@@ -6529,7 +6529,7 @@
     <row r="88">
       <c r="A88" s="47" t="inlineStr">
         <is>
-          <t>MON APR 6 — CALORIES DELIVERED PER PERSON</t>
+          <t>MON JUL 27 — CALORIES DELIVERED PER PERSON</t>
         </is>
       </c>
       <c r="B88" s="47" t="n"/>
@@ -6690,7 +6690,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OHLONE WILDERNESS TRAIL  ·  Bear Can Packing List  ·  April 4–6, 2026</t>
+          <t>OHLONE WILDERNESS TRAIL  ·  Bear Can Packing List  ·  July 25–27, 2026</t>
         </is>
       </c>
     </row>
@@ -6745,7 +6745,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>SATURDAY  APR 4</t>
+          <t>SATURDAY  JUL 25</t>
         </is>
       </c>
     </row>
@@ -7155,7 +7155,7 @@
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>SUNDAY  APR 5</t>
+          <t>SUNDAY  JUL 26</t>
         </is>
       </c>
     </row>
@@ -7751,7 +7751,7 @@
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>MONDAY  APR 6</t>
+          <t>MONDAY  JUL 27</t>
         </is>
       </c>
     </row>
@@ -8041,7 +8041,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Master Shopping List — 19 People · 6 Bear Cans  |  April 4–6, 2026</t>
+          <t>Master Shopping List — 19 People · 6 Bear Cans  |  July 25–27, 2026</t>
         </is>
       </c>
     </row>
@@ -9840,7 +9840,7 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Sat Apr 4</t>
+          <t>Sat Jul 25</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
@@ -9880,7 +9880,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Sat Apr 4</t>
+          <t>Sat Jul 25</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -9920,7 +9920,7 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Sat Apr 4</t>
+          <t>Sat Jul 25</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
@@ -9960,7 +9960,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Sun Apr 5</t>
+          <t>Sun Jul 26</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -10000,7 +10000,7 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Sun Apr 5</t>
+          <t>Sun Jul 26</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
@@ -10040,7 +10040,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Sun Apr 5</t>
+          <t>Sun Jul 26</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -10080,7 +10080,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Sun Apr 5</t>
+          <t>Sun Jul 26</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -10120,7 +10120,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Sun Apr 5</t>
+          <t>Sun Jul 26</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -10160,7 +10160,7 @@
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>Mon Apr 6</t>
+          <t>Mon Jul 27</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
@@ -10200,7 +10200,7 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Mon Apr 6</t>
+          <t>Mon Jul 27</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -10240,7 +10240,7 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Mon Apr 6</t>
+          <t>Mon Jul 27</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Optimize shopping list quantities with dynamic accumulator and update verification script
</commit_message>
<xml_diff>
--- a/spring_hike_menu_19_people.xlsx
+++ b/spring_hike_menu_19_people.xlsx
@@ -1144,7 +1144,7 @@
       </c>
       <c r="J13" s="10" t="inlineStr">
         <is>
-          <t>morales swimming hole side-trip</t>
+          <t>morale swimming hole side-trip</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="J15" s="10" t="inlineStr">
         <is>
-          <t>morales swimming spot; Buck Lake on route</t>
+          <t>morale swimming spot; Buck Lake on route</t>
         </is>
       </c>
     </row>
@@ -1691,19 +1691,19 @@
         </is>
       </c>
       <c r="B35" s="19">
-        <f>SUM('Shopping List'!M$4:M$31)</f>
+        <f>SUM('Shopping List'!M$4:M$32)</f>
         <v/>
       </c>
       <c r="C35" s="19">
-        <f>SUM('Shopping List'!K$4:K$31)</f>
+        <f>SUM('Shopping List'!K$4:K$32)</f>
         <v/>
       </c>
       <c r="D35" s="19">
-        <f>SUM('Shopping List'!L$4:L$31)</f>
+        <f>SUM('Shopping List'!L$4:L$32)</f>
         <v/>
       </c>
       <c r="E35" s="20">
-        <f>SUM('Shopping List'!N$4:N$31)</f>
+        <f>SUM('Shopping List'!N$4:N$32)</f>
         <v/>
       </c>
       <c r="F35" s="10" t="inlineStr">
@@ -1747,19 +1747,19 @@
         </is>
       </c>
       <c r="B37" s="23">
-        <f>SUMPRODUCT('Shopping List'!E$4:E$31,'Shopping List'!O$4:O$31)/16</f>
+        <f>SUMPRODUCT('Shopping List'!E$4:E$32,'Shopping List'!O$4:O$32)/16</f>
         <v/>
       </c>
       <c r="C37" s="23">
-        <f>SUMPRODUCT('Shopping List'!C$4:C$31,'Shopping List'!O$4:O$31)/16</f>
+        <f>SUMPRODUCT('Shopping List'!C$4:C$32,'Shopping List'!O$4:O$32)/16</f>
         <v/>
       </c>
       <c r="D37" s="23">
-        <f>SUMPRODUCT('Shopping List'!D$4:D$31,'Shopping List'!O$4:O$31)/16</f>
+        <f>SUMPRODUCT('Shopping List'!D$4:D$32,'Shopping List'!O$4:O$32)/16</f>
         <v/>
       </c>
       <c r="E37" s="24">
-        <f>SUMPRODUCT(3*'Shopping List'!C$4:C$31+1*'Shopping List'!D$4:D$31+2*'Shopping List'!E$4:E$31,'Shopping List'!O$4:O$31)/16</f>
+        <f>SUMPRODUCT(3*'Shopping List'!C$4:C$32+1*'Shopping List'!D$4:D$32+2*'Shopping List'!E$4:E$32,'Shopping List'!O$4:O$32)/16</f>
         <v/>
       </c>
       <c r="F37" s="10" t="inlineStr">
@@ -1775,19 +1775,19 @@
         </is>
       </c>
       <c r="B38" s="25">
-        <f>SUMPRODUCT('Shopping List'!H$4:H$31,'Shopping List'!O$4:O$31)/16</f>
+        <f>SUMPRODUCT('Shopping List'!H$4:H$32,'Shopping List'!O$4:O$32)/16</f>
         <v/>
       </c>
       <c r="C38" s="25">
-        <f>SUMPRODUCT('Shopping List'!F$4:F$31,'Shopping List'!O$4:O$31)/16</f>
+        <f>SUMPRODUCT('Shopping List'!F$4:F$32,'Shopping List'!O$4:O$32)/16</f>
         <v/>
       </c>
       <c r="D38" s="25">
-        <f>SUMPRODUCT('Shopping List'!G$4:G$31,'Shopping List'!O$4:O$31)/16</f>
+        <f>SUMPRODUCT('Shopping List'!G$4:G$32,'Shopping List'!O$4:O$32)/16</f>
         <v/>
       </c>
       <c r="E38" s="26">
-        <f>SUMPRODUCT(3*'Shopping List'!F$4:F$31+1*'Shopping List'!G$4:G$31+2*'Shopping List'!H$4:H$31,'Shopping List'!O$4:O$31)/16</f>
+        <f>SUMPRODUCT(3*'Shopping List'!F$4:F$32+1*'Shopping List'!G$4:G$32+2*'Shopping List'!H$4:H$32,'Shopping List'!O$4:O$32)/16</f>
         <v/>
       </c>
       <c r="F38" s="7" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>Morale boost lunch stop. Filter all water.</t>
+          <t>morale boost lunch stop. Filter all water.</t>
         </is>
       </c>
     </row>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>morales swimming spot side trip nearby.</t>
+          <t>morale swimming spot side trip nearby.</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>Morale boost meadow camp. Filter water.</t>
+          <t>morale boost meadow camp. Filter water.</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1976,7 @@
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>morales swimming spot. Filter.</t>
+          <t>morale swimming spot. Filter.</t>
         </is>
       </c>
     </row>
@@ -1998,7 +1998,7 @@
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>Morale boost finish. Walk out valley.</t>
+          <t>morale boost finish. Walk out valley.</t>
         </is>
       </c>
     </row>
@@ -13550,7 +13550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q32"/>
+  <dimension ref="A1:Q33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="128" customWidth="1" min="1" max="1"/>
@@ -13693,33 +13693,32 @@
       </c>
       <c r="B4" s="32" t="inlineStr">
         <is>
-          <t>MET-Rx Big100 – Super Cookie Crunch</t>
+          <t>88 Acres Seed + Oat Bars (allergy scout)</t>
         </is>
       </c>
       <c r="C4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="D4" s="33" t="n">
-        <v>8</v>
-      </c>
-      <c r="E4" s="33" t="n">
-        <v>6</v>
-      </c>
-      <c r="F4" s="33" t="n">
-        <v>9</v>
-      </c>
-      <c r="G4" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="H4" s="33" t="n">
-        <v>9</v>
-      </c>
-      <c r="I4" s="33">
-        <f>3*(C4+F4)+1*(D4+G4)+2*(E4+H4)</f>
-        <v/>
-      </c>
       <c r="J4" s="35" t="n">
-        <v>2.19</v>
+        <v>2.4</v>
       </c>
       <c r="K4" s="35">
         <f>(C4+F4)*J4</f>
@@ -13738,7 +13737,7 @@
         <v/>
       </c>
       <c r="O4" s="33" t="n">
-        <v>3.53</v>
+        <v>1.4</v>
       </c>
       <c r="P4" s="36">
         <f>I4*O4</f>
@@ -13746,72 +13745,72 @@
       </c>
       <c r="Q4" s="32" t="inlineStr">
         <is>
-          <t>Bkfst; ⚠ NUT</t>
+          <t>Allergy scout snacks swap</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="33" t="inlineStr">
+      <c r="A5" s="53" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B5" s="32" t="inlineStr">
-        <is>
-          <t>ProBar Meal – Oatmeal Chocolate Chip</t>
-        </is>
-      </c>
-      <c r="C5" s="33" t="n">
+      <c r="B5" s="52" t="inlineStr">
+        <is>
+          <t>Adults: own coffee / tea</t>
+        </is>
+      </c>
+      <c r="C5" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="53" t="n">
         <v>6</v>
       </c>
-      <c r="D5" s="33" t="n">
-        <v>8</v>
-      </c>
-      <c r="E5" s="33" t="n">
-        <v>6</v>
-      </c>
-      <c r="F5" s="33" t="n">
+      <c r="F5" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="53" t="n">
         <v>9</v>
       </c>
-      <c r="G5" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="H5" s="33" t="n">
-        <v>9</v>
-      </c>
-      <c r="I5" s="33">
+      <c r="I5" s="53">
         <f>3*(C5+F5)+1*(D5+G5)+2*(E5+H5)</f>
         <v/>
       </c>
-      <c r="J5" s="35" t="n">
-        <v>2.99</v>
-      </c>
-      <c r="K5" s="35">
+      <c r="J5" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="55">
         <f>(C5+F5)*J5</f>
         <v/>
       </c>
-      <c r="L5" s="35">
+      <c r="L5" s="55">
         <f>(D5+G5)*J5</f>
         <v/>
       </c>
-      <c r="M5" s="35">
+      <c r="M5" s="55">
         <f>(E5+H5)*J5</f>
         <v/>
       </c>
-      <c r="N5" s="35">
+      <c r="N5" s="55">
         <f>I5*J5</f>
         <v/>
       </c>
-      <c r="O5" s="33" t="n">
-        <v>3</v>
-      </c>
-      <c r="P5" s="36">
+      <c r="O5" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="56">
         <f>I5*O5</f>
         <v/>
       </c>
-      <c r="Q5" s="32" t="inlineStr">
-        <is>
-          <t>Bkfst &amp; Lunch; ⚠ NUT (cashews)</t>
+      <c r="Q5" s="52" t="inlineStr">
+        <is>
+          <t>Adults only ★</t>
         </is>
       </c>
     </row>
@@ -13823,33 +13822,33 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Peak Refuel – Beef Pasta Marinara</t>
+          <t>Backpacker's Pantry – Crème Brûlée</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
         <v>4</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>2</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I6" s="6">
         <f>3*(C6+F6)+1*(D6+G6)+2*(E6+H6)</f>
         <v/>
       </c>
       <c r="J6" s="41" t="n">
-        <v>7.49</v>
+        <v>8.99</v>
       </c>
       <c r="K6" s="41">
         <f>(C6+F6)*J6</f>
@@ -13868,7 +13867,7 @@
         <v/>
       </c>
       <c r="O6" s="6" t="n">
-        <v>3.2</v>
+        <v>2.26</v>
       </c>
       <c r="P6" s="42">
         <f>I6*O6</f>
@@ -13876,7 +13875,7 @@
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>Dinner (1.5 svgs/pouch)</t>
+          <t>Buddy-pair shares pouch</t>
         </is>
       </c>
     </row>
@@ -13886,25 +13885,25 @@
           <t>☐</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Peak Refuel – Beef Stroganoff</t>
+      <c r="B7" s="66" t="inlineStr">
+        <is>
+          <t>Banana Chips (1 oz)</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E7" s="9" t="n">
         <v>3</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H7" s="9" t="n">
         <v>3</v>
@@ -13914,7 +13913,7 @@
         <v/>
       </c>
       <c r="J7" s="38" t="n">
-        <v>7.49</v>
+        <v>0.45</v>
       </c>
       <c r="K7" s="38">
         <f>(C7+F7)*J7</f>
@@ -13933,7 +13932,7 @@
         <v/>
       </c>
       <c r="O7" s="9" t="n">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="P7" s="39">
         <f>I7*O7</f>
@@ -13941,7 +13940,7 @@
       </c>
       <c r="Q7" s="10" t="inlineStr">
         <is>
-          <t>Dinner (1.5 svgs/pouch)</t>
+          <t>Nut-free ✓</t>
         </is>
       </c>
     </row>
@@ -13951,35 +13950,35 @@
           <t>☐</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Backpacker's Pantry – Crème Brûlée</t>
+      <c r="B8" s="66" t="inlineStr">
+        <is>
+          <t>Chicken of the Sea Shredded Chicken Pouch</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>4</v>
       </c>
       <c r="E8" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" s="6" t="n">
-        <v>2</v>
-      </c>
       <c r="H8" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I8" s="6">
         <f>3*(C8+F8)+1*(D8+G8)+2*(E8+H8)</f>
         <v/>
       </c>
       <c r="J8" s="41" t="n">
-        <v>8.99</v>
+        <v>2.29</v>
       </c>
       <c r="K8" s="41">
         <f>(C8+F8)*J8</f>
@@ -13998,7 +13997,7 @@
         <v/>
       </c>
       <c r="O8" s="6" t="n">
-        <v>2.26</v>
+        <v>2.5</v>
       </c>
       <c r="P8" s="42">
         <f>I8*O8</f>
@@ -14006,7 +14005,7 @@
       </c>
       <c r="Q8" s="7" t="inlineStr">
         <is>
-          <t>Dessert (shares pouch)</t>
+          <t>No cook; nut-free ✓</t>
         </is>
       </c>
     </row>
@@ -14018,33 +14017,33 @@
       </c>
       <c r="B9" s="32" t="inlineStr">
         <is>
-          <t>Justin's Dark Chocolate Peanut Butter Cups</t>
+          <t>Clif Bar – Crunchy PB</t>
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G9" s="33" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H9" s="33" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I9" s="33">
         <f>3*(C9+F9)+1*(D9+G9)+2*(E9+H9)</f>
         <v/>
       </c>
       <c r="J9" s="35" t="n">
-        <v>1.49</v>
+        <v>1.29</v>
       </c>
       <c r="K9" s="35">
         <f>(C9+F9)*J9</f>
@@ -14063,7 +14062,7 @@
         <v/>
       </c>
       <c r="O9" s="33" t="n">
-        <v>1.41</v>
+        <v>2.4</v>
       </c>
       <c r="P9" s="36">
         <f>I9*O9</f>
@@ -14071,72 +14070,72 @@
       </c>
       <c r="Q9" s="32" t="inlineStr">
         <is>
-          <t>Dessert; ⚠ NUT</t>
+          <t>Lunch snack; ⚠ NUT</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="33" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B10" s="66" t="inlineStr">
-        <is>
-          <t>Columbus Hard Salami (sliced packet)</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="I10" s="6">
+      <c r="B10" s="32" t="inlineStr">
+        <is>
+          <t>Clif Builder's Bar (adult supplement)</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" s="33">
         <f>3*(C10+F10)+1*(D10+G10)+2*(E10+H10)</f>
         <v/>
       </c>
-      <c r="J10" s="41" t="n">
-        <v>2.99</v>
-      </c>
-      <c r="K10" s="41">
+      <c r="J10" s="35" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="K10" s="35">
         <f>(C10+F10)*J10</f>
         <v/>
       </c>
-      <c r="L10" s="41">
+      <c r="L10" s="35">
         <f>(D10+G10)*J10</f>
         <v/>
       </c>
-      <c r="M10" s="41">
+      <c r="M10" s="35">
         <f>(E10+H10)*J10</f>
         <v/>
       </c>
-      <c r="N10" s="41">
+      <c r="N10" s="35">
         <f>I10*J10</f>
         <v/>
       </c>
-      <c r="O10" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P10" s="42">
+      <c r="O10" s="33" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P10" s="36">
         <f>I10*O10</f>
         <v/>
       </c>
-      <c r="Q10" s="7" t="inlineStr">
-        <is>
-          <t>Lunch; 1/person</t>
+      <c r="Q10" s="32" t="inlineStr">
+        <is>
+          <t>Adults only ★; ⚠ NUT</t>
         </is>
       </c>
     </row>
@@ -14146,9 +14145,9 @@
           <t>☐</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Wasa Crisp'n Light Crackerbread</t>
+      <c r="B11" s="66" t="inlineStr">
+        <is>
+          <t>Columbus Hard Salami (sliced packet)</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
@@ -14174,7 +14173,7 @@
         <v/>
       </c>
       <c r="J11" s="38" t="n">
-        <v>0.5</v>
+        <v>2.99</v>
       </c>
       <c r="K11" s="38">
         <f>(C11+F11)*J11</f>
@@ -14193,7 +14192,7 @@
         <v/>
       </c>
       <c r="O11" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P11" s="39">
         <f>I11*O11</f>
@@ -14201,7 +14200,7 @@
       </c>
       <c r="Q11" s="10" t="inlineStr">
         <is>
-          <t>Lunch side</t>
+          <t>Lunch; 1/person; nut-free</t>
         </is>
       </c>
     </row>
@@ -14213,33 +14212,33 @@
       </c>
       <c r="B12" s="66" t="inlineStr">
         <is>
-          <t>Chicken of the Sea Shredded Chicken Pouch</t>
+          <t>Gatorade Powder Pack</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="I12" s="6">
         <f>3*(C12+F12)+1*(D12+G12)+2*(E12+H12)</f>
         <v/>
       </c>
       <c r="J12" s="41" t="n">
-        <v>2.29</v>
+        <v>0.38</v>
       </c>
       <c r="K12" s="41">
         <f>(C12+F12)*J12</f>
@@ -14258,7 +14257,7 @@
         <v/>
       </c>
       <c r="O12" s="6" t="n">
-        <v>2.5</v>
+        <v>1.23</v>
       </c>
       <c r="P12" s="42">
         <f>I12*O12</f>
@@ -14266,72 +14265,71 @@
       </c>
       <c r="Q12" s="7" t="inlineStr">
         <is>
-          <t>Lunch; 1/person</t>
+          <t>Electrolytes</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="33" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B13" s="66" t="inlineStr">
-        <is>
-          <t>Mission Street Taco Flour Tortillas</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="D13" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="F13" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="H13" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="I13" s="9">
-        <f>3*(C13+F13)+1*(D13+G13)+2*(E13+H13)</f>
-        <v/>
-      </c>
-      <c r="J13" s="38" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="K13" s="38">
+      <c r="B13" s="32" t="inlineStr">
+        <is>
+          <t>Honey Stinger Gold Waffle (allergy scout)</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="J13" s="35" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="K13" s="35">
         <f>(C13+F13)*J13</f>
         <v/>
       </c>
-      <c r="L13" s="38">
+      <c r="L13" s="35">
         <f>(D13+G13)*J13</f>
         <v/>
       </c>
-      <c r="M13" s="38">
+      <c r="M13" s="35">
         <f>(E13+H13)*J13</f>
         <v/>
       </c>
-      <c r="N13" s="38">
+      <c r="N13" s="35">
         <f>I13*J13</f>
         <v/>
       </c>
-      <c r="O13" s="9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P13" s="39">
+      <c r="O13" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" s="36">
         <f>I13*O13</f>
         <v/>
       </c>
-      <c r="Q13" s="10" t="inlineStr">
-        <is>
-          <t>lunch + dinner wraps</t>
+      <c r="Q13" s="32" t="inlineStr">
+        <is>
+          <t>Allergy scout dessert swap</t>
         </is>
       </c>
     </row>
@@ -14341,35 +14339,35 @@
           <t>☐</t>
         </is>
       </c>
-      <c r="B14" s="66" t="inlineStr">
-        <is>
-          <t>Tillamook Cheddar Cheese Packets</t>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Idahoan Mashed Potatoes – Butter &amp; Herb</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="I14" s="6">
         <f>3*(C14+F14)+1*(D14+G14)+2*(E14+H14)</f>
         <v/>
       </c>
       <c r="J14" s="41" t="n">
-        <v>0.75</v>
+        <v>0.98</v>
       </c>
       <c r="K14" s="41">
         <f>(C14+F14)*J14</f>
@@ -14388,7 +14386,7 @@
         <v/>
       </c>
       <c r="O14" s="6" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="P14" s="42">
         <f>I14*O14</f>
@@ -14396,7 +14394,7 @@
       </c>
       <c r="Q14" s="7" t="inlineStr">
         <is>
-          <t>lunch + dinner side</t>
+          <t>Dinner side</t>
         </is>
       </c>
     </row>
@@ -14466,67 +14464,67 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="33" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Idahoan Mashed Potatoes – Butter &amp; Herb</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D16" s="6" t="n">
+      <c r="B16" s="32" t="inlineStr">
+        <is>
+          <t>Justin's Dark Chocolate Peanut Butter Cups</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="33" t="n">
         <v>4</v>
       </c>
-      <c r="E16" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="F16" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="G16" s="6" t="n">
+      <c r="E16" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="33" t="n">
         <v>4</v>
       </c>
-      <c r="H16" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="I16" s="6">
+      <c r="H16" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="I16" s="33">
         <f>3*(C16+F16)+1*(D16+G16)+2*(E16+H16)</f>
         <v/>
       </c>
-      <c r="J16" s="41" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="K16" s="41">
+      <c r="J16" s="35" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="K16" s="35">
         <f>(C16+F16)*J16</f>
         <v/>
       </c>
-      <c r="L16" s="41">
+      <c r="L16" s="35">
         <f>(D16+G16)*J16</f>
         <v/>
       </c>
-      <c r="M16" s="41">
+      <c r="M16" s="35">
         <f>(E16+H16)*J16</f>
         <v/>
       </c>
-      <c r="N16" s="41">
+      <c r="N16" s="35">
         <f>I16*J16</f>
         <v/>
       </c>
-      <c r="O16" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P16" s="42">
+      <c r="O16" s="33" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="P16" s="36">
         <f>I16*O16</f>
         <v/>
       </c>
-      <c r="Q16" s="7" t="inlineStr">
-        <is>
-          <t>Dinner side</t>
+      <c r="Q16" s="32" t="inlineStr">
+        <is>
+          <t>1 packet/person; ⚠ NUT</t>
         </is>
       </c>
     </row>
@@ -14538,33 +14536,33 @@
       </c>
       <c r="B17" s="32" t="inlineStr">
         <is>
-          <t>Kind – Peanut Butter Dark Chocolate Bar</t>
+          <t>Justin's PB Squeeze (adult supplement)</t>
         </is>
       </c>
       <c r="C17" s="33" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D17" s="33" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E17" s="33" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F17" s="33" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G17" s="33" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H17" s="33" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I17" s="33">
         <f>3*(C17+F17)+1*(D17+G17)+2*(E17+H17)</f>
         <v/>
       </c>
       <c r="J17" s="35" t="n">
-        <v>1.04</v>
+        <v>1.49</v>
       </c>
       <c r="K17" s="35">
         <f>(C17+F17)*J17</f>
@@ -14583,7 +14581,7 @@
         <v/>
       </c>
       <c r="O17" s="33" t="n">
-        <v>1.4</v>
+        <v>1.15</v>
       </c>
       <c r="P17" s="36">
         <f>I17*O17</f>
@@ -14591,7 +14589,7 @@
       </c>
       <c r="Q17" s="32" t="inlineStr">
         <is>
-          <t>Snacks; ⚠ NUT</t>
+          <t>Adults only ★; ⚠ NUT</t>
         </is>
       </c>
     </row>
@@ -14607,22 +14605,22 @@
         </is>
       </c>
       <c r="C18" s="33" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D18" s="33" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E18" s="33" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F18" s="33" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G18" s="33" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H18" s="33" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I18" s="33">
         <f>3*(C18+F18)+1*(D18+G18)+2*(E18+H18)</f>
@@ -14656,7 +14654,7 @@
       </c>
       <c r="Q18" s="32" t="inlineStr">
         <is>
-          <t>Snacks; ⚠ NUT</t>
+          <t>⚠ NUT: swap → 88 Acres bar</t>
         </is>
       </c>
     </row>
@@ -14672,22 +14670,22 @@
         </is>
       </c>
       <c r="C19" s="33" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D19" s="33" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E19" s="33" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F19" s="33" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G19" s="33" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H19" s="33" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I19" s="33">
         <f>3*(C19+F19)+1*(D19+G19)+2*(E19+H19)</f>
@@ -14721,72 +14719,72 @@
       </c>
       <c r="Q19" s="32" t="inlineStr">
         <is>
-          <t>Snacks; ⚠ NUT</t>
+          <t>⚠ NUT: swap → 88 Acres bar</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="33" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B20" s="66" t="inlineStr">
-        <is>
-          <t>Krave Sea Salt Original Beef Jerky</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="D20" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="E20" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="F20" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G20" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="H20" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="I20" s="6">
+      <c r="B20" s="32" t="inlineStr">
+        <is>
+          <t>Kind – Peanut Butter Dark Chocolate Bar</t>
+        </is>
+      </c>
+      <c r="C20" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="33" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" s="33" t="n">
+        <v>4</v>
+      </c>
+      <c r="H20" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="I20" s="33">
         <f>3*(C20+F20)+1*(D20+G20)+2*(E20+H20)</f>
         <v/>
       </c>
-      <c r="J20" s="41" t="n">
-        <v>2.19</v>
-      </c>
-      <c r="K20" s="41">
+      <c r="J20" s="35" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="K20" s="35">
         <f>(C20+F20)*J20</f>
         <v/>
       </c>
-      <c r="L20" s="41">
+      <c r="L20" s="35">
         <f>(D20+G20)*J20</f>
         <v/>
       </c>
-      <c r="M20" s="41">
+      <c r="M20" s="35">
         <f>(E20+H20)*J20</f>
         <v/>
       </c>
-      <c r="N20" s="41">
+      <c r="N20" s="35">
         <f>I20*J20</f>
         <v/>
       </c>
-      <c r="O20" s="6" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="P20" s="42">
+      <c r="O20" s="33" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="P20" s="36">
         <f>I20*O20</f>
         <v/>
       </c>
-      <c r="Q20" s="7" t="inlineStr">
-        <is>
-          <t>Snacks</t>
+      <c r="Q20" s="32" t="inlineStr">
+        <is>
+          <t>⚠ NUT: swap → 88 Acres bar</t>
         </is>
       </c>
     </row>
@@ -14798,33 +14796,33 @@
       </c>
       <c r="B21" s="66" t="inlineStr">
         <is>
-          <t>Gatorade Powder Pack</t>
+          <t>Krave Sea Salt Original Beef Jerky</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D21" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="D21" s="9" t="n">
-        <v>16</v>
-      </c>
       <c r="E21" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="G21" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="F21" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="G21" s="9" t="n">
-        <v>16</v>
-      </c>
       <c r="H21" s="9" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="I21" s="9">
         <f>3*(C21+F21)+1*(D21+G21)+2*(E21+H21)</f>
         <v/>
       </c>
       <c r="J21" s="38" t="n">
-        <v>0.38</v>
+        <v>2.19</v>
       </c>
       <c r="K21" s="38">
         <f>(C21+F21)*J21</f>
@@ -14843,7 +14841,7 @@
         <v/>
       </c>
       <c r="O21" s="9" t="n">
-        <v>1.23</v>
+        <v>1.48</v>
       </c>
       <c r="P21" s="39">
         <f>I21*O21</f>
@@ -14851,7 +14849,7 @@
       </c>
       <c r="Q21" s="10" t="inlineStr">
         <is>
-          <t>Snacks</t>
+          <t>Safe for nut allergy ✓</t>
         </is>
       </c>
     </row>
@@ -14863,17 +14861,17 @@
       </c>
       <c r="B22" s="32" t="inlineStr">
         <is>
-          <t>Clif Bar – Crunchy PB</t>
+          <t>MET-Rx Big100 – Super Cookie Crunch</t>
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D22" s="33" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E22" s="33" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F22" s="33" t="n">
         <v>6</v>
@@ -14889,7 +14887,7 @@
         <v/>
       </c>
       <c r="J22" s="35" t="n">
-        <v>1.29</v>
+        <v>2.19</v>
       </c>
       <c r="K22" s="35">
         <f>(C22+F22)*J22</f>
@@ -14908,7 +14906,7 @@
         <v/>
       </c>
       <c r="O22" s="33" t="n">
-        <v>2.4</v>
+        <v>3.53</v>
       </c>
       <c r="P22" s="36">
         <f>I22*O22</f>
@@ -14916,72 +14914,72 @@
       </c>
       <c r="Q22" s="32" t="inlineStr">
         <is>
-          <t>Lunch snack; ⚠ NUT</t>
+          <t>Bkfst · ⚠ NUT</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="33" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B23" s="32" t="inlineStr">
-        <is>
-          <t>Clif Builder's Bar (adult supplement)</t>
-        </is>
-      </c>
-      <c r="C23" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="33" t="n">
-        <v>9</v>
-      </c>
-      <c r="F23" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="33" t="n">
-        <v>9</v>
-      </c>
-      <c r="I23" s="33">
+      <c r="B23" s="66" t="inlineStr">
+        <is>
+          <t>Mission Street Taco Flour Tortillas</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="H23" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="I23" s="9">
         <f>3*(C23+F23)+1*(D23+G23)+2*(E23+H23)</f>
         <v/>
       </c>
-      <c r="J23" s="35" t="n">
-        <v>2.17</v>
-      </c>
-      <c r="K23" s="35">
+      <c r="J23" s="38" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K23" s="38">
         <f>(C23+F23)*J23</f>
         <v/>
       </c>
-      <c r="L23" s="35">
+      <c r="L23" s="38">
         <f>(D23+G23)*J23</f>
         <v/>
       </c>
-      <c r="M23" s="35">
+      <c r="M23" s="38">
         <f>(E23+H23)*J23</f>
         <v/>
       </c>
-      <c r="N23" s="35">
+      <c r="N23" s="38">
         <f>I23*J23</f>
         <v/>
       </c>
-      <c r="O23" s="33" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="P23" s="36">
+      <c r="O23" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P23" s="39">
         <f>I23*O23</f>
         <v/>
       </c>
-      <c r="Q23" s="32" t="inlineStr">
-        <is>
-          <t>Adults ★; ⚠ NUT</t>
+      <c r="Q23" s="10" t="inlineStr">
+        <is>
+          <t>2/person; nut-free ✓</t>
         </is>
       </c>
     </row>
@@ -14993,7 +14991,7 @@
       </c>
       <c r="B24" s="32" t="inlineStr">
         <is>
-          <t>Justin's PB Squeeze (adult supplement)</t>
+          <t>Once Again Organic Sunflower Butter Squeeze</t>
         </is>
       </c>
       <c r="C24" s="33" t="n">
@@ -15003,7 +15001,7 @@
         <v>0</v>
       </c>
       <c r="E24" s="33" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F24" s="33" t="n">
         <v>0</v>
@@ -15012,14 +15010,13 @@
         <v>0</v>
       </c>
       <c r="H24" s="33" t="n">
-        <v>9</v>
-      </c>
-      <c r="I24" s="33">
-        <f>3*(C24+F24)+1*(D24+G24)+2*(E24+H24)</f>
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="I24" s="33" t="n">
+        <v>4</v>
       </c>
       <c r="J24" s="35" t="n">
-        <v>1.49</v>
+        <v>1.5</v>
       </c>
       <c r="K24" s="35">
         <f>(C24+F24)*J24</f>
@@ -15046,7 +15043,7 @@
       </c>
       <c r="Q24" s="32" t="inlineStr">
         <is>
-          <t>Adults ★; ⚠ NUT</t>
+          <t>Allergy scout PB swap</t>
         </is>
       </c>
     </row>
@@ -15056,35 +15053,35 @@
           <t>☐</t>
         </is>
       </c>
-      <c r="B25" s="66" t="inlineStr">
-        <is>
-          <t>Swiss Miss Hot Chocolate</t>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Peak Refuel – Beef Pasta Marinara</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I25" s="9">
         <f>3*(C25+F25)+1*(D25+G25)+2*(E25+H25)</f>
         <v/>
       </c>
       <c r="J25" s="38" t="n">
-        <v>0.38</v>
+        <v>7.49</v>
       </c>
       <c r="K25" s="38">
         <f>(C25+F25)*J25</f>
@@ -15103,7 +15100,7 @@
         <v/>
       </c>
       <c r="O25" s="9" t="n">
-        <v>0.73</v>
+        <v>3.2</v>
       </c>
       <c r="P25" s="39">
         <f>I25*O25</f>
@@ -15111,7 +15108,7 @@
       </c>
       <c r="Q25" s="10" t="inlineStr">
         <is>
-          <t>Scouts only</t>
+          <t>Sat dinner (1.5 svgs/pouch)</t>
         </is>
       </c>
     </row>
@@ -15123,33 +15120,33 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Peak Refuel – Fudge Brownie Bites</t>
+          <t>Peak Refuel – Beef Stroganoff</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F26" s="6" t="n">
         <v>2</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I26" s="6">
         <f>3*(C26+F26)+1*(D26+G26)+2*(E26+H26)</f>
         <v/>
       </c>
       <c r="J26" s="41" t="n">
-        <v>4.99</v>
+        <v>7.49</v>
       </c>
       <c r="K26" s="41">
         <f>(C26+F26)*J26</f>
@@ -15168,7 +15165,7 @@
         <v/>
       </c>
       <c r="O26" s="6" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="P26" s="42">
         <f>I26*O26</f>
@@ -15176,7 +15173,7 @@
       </c>
       <c r="Q26" s="7" t="inlineStr">
         <is>
-          <t>Snacks</t>
+          <t>Sun dinner (1.5 svgs/pouch)</t>
         </is>
       </c>
     </row>
@@ -15188,33 +15185,33 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Trader Joe's Dried Mango Slices (1 oz)</t>
+          <t>Peak Refuel – Fudge Brownie Bites</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E27" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I27" s="9">
         <f>3*(C27+F27)+1*(D27+G27)+2*(E27+H27)</f>
         <v/>
       </c>
       <c r="J27" s="38" t="n">
-        <v>0.55</v>
+        <v>4.99</v>
       </c>
       <c r="K27" s="38">
         <f>(C27+F27)*J27</f>
@@ -15233,7 +15230,7 @@
         <v/>
       </c>
       <c r="O27" s="9" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="P27" s="39">
         <f>I27*O27</f>
@@ -15241,304 +15238,372 @@
       </c>
       <c r="Q27" s="10" t="inlineStr">
         <is>
-          <t>Snacks</t>
+          <t>Buddy-pair shares pouch</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="33" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B28" s="66" t="inlineStr">
-        <is>
-          <t>Banana Chips (1 oz)</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D28" s="6" t="n">
+      <c r="B28" s="32" t="inlineStr">
+        <is>
+          <t>ProBar Meal – Oatmeal Chocolate Chip</t>
+        </is>
+      </c>
+      <c r="C28" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="D28" s="33" t="n">
+        <v>8</v>
+      </c>
+      <c r="E28" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="G28" s="33" t="n">
+        <v>8</v>
+      </c>
+      <c r="H28" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="I28" s="33">
+        <f>3*(C28+F28)+1*(D28+G28)+2*(E28+H28)</f>
+        <v/>
+      </c>
+      <c r="J28" s="35" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="K28" s="35">
+        <f>(C28+F28)*J28</f>
+        <v/>
+      </c>
+      <c r="L28" s="35">
+        <f>(D28+G28)*J28</f>
+        <v/>
+      </c>
+      <c r="M28" s="35">
+        <f>(E28+H28)*J28</f>
+        <v/>
+      </c>
+      <c r="N28" s="35">
+        <f>I28*J28</f>
+        <v/>
+      </c>
+      <c r="O28" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="P28" s="36">
+        <f>I28*O28</f>
+        <v/>
+      </c>
+      <c r="Q28" s="32" t="inlineStr">
+        <is>
+          <t>Lunch · ⚠ NUT (cashews)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B29" s="66" t="inlineStr">
+        <is>
+          <t>Swiss Miss Hot Chocolate</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="9">
+        <f>3*(C29+F29)+1*(D29+G29)+2*(E29+H29)</f>
+        <v/>
+      </c>
+      <c r="J29" s="38" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="K29" s="38">
+        <f>(C29+F29)*J29</f>
+        <v/>
+      </c>
+      <c r="L29" s="38">
+        <f>(D29+G29)*J29</f>
+        <v/>
+      </c>
+      <c r="M29" s="38">
+        <f>(E29+H29)*J29</f>
+        <v/>
+      </c>
+      <c r="N29" s="38">
+        <f>I29*J29</f>
+        <v/>
+      </c>
+      <c r="O29" s="9" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="P29" s="39">
+        <f>I29*O29</f>
+        <v/>
+      </c>
+      <c r="Q29" s="10" t="inlineStr">
+        <is>
+          <t>Scouts only (2 packets/person)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B30" s="66" t="inlineStr">
+        <is>
+          <t>Tillamook Cheddar Cheese Packets</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="I30" s="6">
+        <f>3*(C30+F30)+1*(D30+G30)+2*(E30+H30)</f>
+        <v/>
+      </c>
+      <c r="J30" s="41" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K30" s="41">
+        <f>(C30+F30)*J30</f>
+        <v/>
+      </c>
+      <c r="L30" s="41">
+        <f>(D30+G30)*J30</f>
+        <v/>
+      </c>
+      <c r="M30" s="41">
+        <f>(E30+H30)*J30</f>
+        <v/>
+      </c>
+      <c r="N30" s="41">
+        <f>I30*J30</f>
+        <v/>
+      </c>
+      <c r="O30" s="6" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="P30" s="42">
+        <f>I30*O30</f>
+        <v/>
+      </c>
+      <c r="Q30" s="7" t="inlineStr">
+        <is>
+          <t>2/person; nut-free ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Trader Joe's Dried Mango Slices (1 oz)</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E28" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="F28" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="G28" s="6" t="n">
+      <c r="E31" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G31" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="H28" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="I28" s="6">
-        <f>3*(C28+F28)+1*(D28+G28)+2*(E28+H28)</f>
-        <v/>
-      </c>
-      <c r="J28" s="41" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="K28" s="41">
-        <f>(C28+F28)*J28</f>
-        <v/>
-      </c>
-      <c r="L28" s="41">
-        <f>(D28+G28)*J28</f>
-        <v/>
-      </c>
-      <c r="M28" s="41">
-        <f>(E28+H28)*J28</f>
-        <v/>
-      </c>
-      <c r="N28" s="41">
-        <f>I28*J28</f>
-        <v/>
-      </c>
-      <c r="O28" s="6" t="n">
+      <c r="H31" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I31" s="9">
+        <f>3*(C31+F31)+1*(D31+G31)+2*(E31+H31)</f>
+        <v/>
+      </c>
+      <c r="J31" s="38" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="K31" s="38">
+        <f>(C31+F31)*J31</f>
+        <v/>
+      </c>
+      <c r="L31" s="38">
+        <f>(D31+G31)*J31</f>
+        <v/>
+      </c>
+      <c r="M31" s="38">
+        <f>(E31+H31)*J31</f>
+        <v/>
+      </c>
+      <c r="N31" s="38">
+        <f>I31*J31</f>
+        <v/>
+      </c>
+      <c r="O31" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="P28" s="42">
-        <f>I28*O28</f>
-        <v/>
-      </c>
-      <c r="Q28" s="7" t="inlineStr">
-        <is>
-          <t>Snacks</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="33" t="inlineStr">
+      <c r="P31" s="39">
+        <f>I31*O31</f>
+        <v/>
+      </c>
+      <c r="Q31" s="10" t="inlineStr">
+        <is>
+          <t>TJ's — Sat snack · nut-free ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B29" s="32" t="inlineStr">
-        <is>
-          <t>88 Acres Seed + Oat Bars (allergy scout)</t>
-        </is>
-      </c>
-      <c r="C29" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="33" t="n">
-        <v>6</v>
-      </c>
-      <c r="J29" s="35" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="K29" s="35">
-        <f>(C29+F29)*J29</f>
-        <v/>
-      </c>
-      <c r="L29" s="35">
-        <f>(D29+G29)*J29</f>
-        <v/>
-      </c>
-      <c r="M29" s="35">
-        <f>(E29+H29)*J29</f>
-        <v/>
-      </c>
-      <c r="N29" s="35">
-        <f>I29*J29</f>
-        <v/>
-      </c>
-      <c r="O29" s="33" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="P29" s="36">
-        <f>I29*O29</f>
-        <v/>
-      </c>
-      <c r="Q29" s="32" t="inlineStr">
-        <is>
-          <t>Allergy scout snacks swap</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="33" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B30" s="32" t="inlineStr">
-        <is>
-          <t>Once Again Organic Sunflower Butter Squeeze</t>
-        </is>
-      </c>
-      <c r="C30" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="33" t="n">
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Wasa Crisp'n Light Crackerbread</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="J30" s="35" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="K30" s="35">
-        <f>(C30+F30)*J30</f>
-        <v/>
-      </c>
-      <c r="L30" s="35">
-        <f>(D30+G30)*J30</f>
-        <v/>
-      </c>
-      <c r="M30" s="35">
-        <f>(E30+H30)*J30</f>
-        <v/>
-      </c>
-      <c r="N30" s="35">
-        <f>I30*J30</f>
-        <v/>
-      </c>
-      <c r="O30" s="33" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="P30" s="36">
-        <f>I30*O30</f>
-        <v/>
-      </c>
-      <c r="Q30" s="32" t="inlineStr">
-        <is>
-          <t>Allergy scout PB swap</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="33" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B31" s="32" t="inlineStr">
-        <is>
-          <t>Honey Stinger Gold Waffle (allergy scout)</t>
-        </is>
-      </c>
-      <c r="C31" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="33" t="n">
-        <v>5</v>
-      </c>
-      <c r="J31" s="35" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="K31" s="35">
-        <f>(C31+F31)*J31</f>
-        <v/>
-      </c>
-      <c r="L31" s="35">
-        <f>(D31+G31)*J31</f>
-        <v/>
-      </c>
-      <c r="M31" s="35">
-        <f>(E31+H31)*J31</f>
-        <v/>
-      </c>
-      <c r="N31" s="35">
-        <f>I31*J31</f>
-        <v/>
-      </c>
-      <c r="O31" s="33" t="n">
+      <c r="E32" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I32" s="6">
+        <f>3*(C32+F32)+1*(D32+G32)+2*(E32+H32)</f>
+        <v/>
+      </c>
+      <c r="J32" s="41" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K32" s="41">
+        <f>(C32+F32)*J32</f>
+        <v/>
+      </c>
+      <c r="L32" s="41">
+        <f>(D32+G32)*J32</f>
+        <v/>
+      </c>
+      <c r="M32" s="41">
+        <f>(E32+H32)*J32</f>
+        <v/>
+      </c>
+      <c r="N32" s="41">
+        <f>I32*J32</f>
+        <v/>
+      </c>
+      <c r="O32" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="P31" s="36">
-        <f>I31*O31</f>
-        <v/>
-      </c>
-      <c r="Q31" s="32" t="inlineStr">
-        <is>
-          <t>Allergy scout dessert swap</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="67" t="n"/>
-      <c r="B32" s="67" t="inlineStr">
+      <c r="P32" s="42">
+        <f>I32*O32</f>
+        <v/>
+      </c>
+      <c r="Q32" s="7" t="inlineStr">
+        <is>
+          <t>Lunch side</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="67" t="n"/>
+      <c r="B33" s="67" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="C32" s="67" t="n"/>
-      <c r="D32" s="67" t="n"/>
-      <c r="E32" s="67" t="n"/>
-      <c r="F32" s="67" t="n"/>
-      <c r="G32" s="67" t="n"/>
-      <c r="H32" s="67" t="n"/>
-      <c r="I32" s="67" t="n"/>
-      <c r="J32" s="67" t="n"/>
-      <c r="K32" s="68">
-        <f>SUM(K4:K31)</f>
-        <v/>
-      </c>
-      <c r="L32" s="68">
-        <f>SUM(L4:L31)</f>
-        <v/>
-      </c>
-      <c r="M32" s="68">
-        <f>SUM(M4:M31)</f>
-        <v/>
-      </c>
-      <c r="N32" s="68">
-        <f>SUM(N4:N31)</f>
-        <v/>
-      </c>
-      <c r="O32" s="67" t="n"/>
-      <c r="P32" s="69">
-        <f>SUM(P4:P31)</f>
-        <v/>
-      </c>
-      <c r="Q32" s="67" t="n"/>
+      <c r="C33" s="67" t="n"/>
+      <c r="D33" s="67" t="n"/>
+      <c r="E33" s="67" t="n"/>
+      <c r="F33" s="67" t="n"/>
+      <c r="G33" s="67" t="n"/>
+      <c r="H33" s="67" t="n"/>
+      <c r="I33" s="67" t="n"/>
+      <c r="J33" s="67" t="n"/>
+      <c r="K33" s="68">
+        <f>SUM(K4:K32)</f>
+        <v/>
+      </c>
+      <c r="L33" s="68">
+        <f>SUM(L4:L32)</f>
+        <v/>
+      </c>
+      <c r="M33" s="68">
+        <f>SUM(M4:M32)</f>
+        <v/>
+      </c>
+      <c r="N33" s="68">
+        <f>SUM(N4:N32)</f>
+        <v/>
+      </c>
+      <c r="O33" s="67" t="n"/>
+      <c r="P33" s="69">
+        <f>SUM(P4:P32)</f>
+        <v/>
+      </c>
+      <c r="Q33" s="67" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15560,7 +15625,7 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16851,7 +16916,7 @@
       </c>
       <c r="G47" s="10" t="inlineStr">
         <is>
-          <t>morales afternoon snack; nut-free</t>
+          <t>morale afternoon snack; nut-free</t>
         </is>
       </c>
     </row>
@@ -18522,7 +18587,7 @@
       </c>
       <c r="G104" s="7" t="inlineStr">
         <is>
-          <t>morales afternoon snack; nut-free</t>
+          <t>morale afternoon snack; nut-free</t>
         </is>
       </c>
     </row>

</xml_diff>